<commit_message>
Sync T01 gameplay, map encounters and UI updates
</commit_message>
<xml_diff>
--- a/output/spreadsheet/t01-02-状态与器具控制词典-260928.xlsx
+++ b/output/spreadsheet/t01-02-状态与器具控制词典-260928.xlsx
@@ -63045,7 +63045,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>累积到第10个时生成独立雷盾，并参与内鸣。</t>
+          <t>Buff，本身无效果，每累积10层生成1层雷盾。</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -63060,7 +63060,7 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>核心01 §1.5、§5.30～5.36</t>
+          <t>核心01 §1.5、§1.24、§5.30～5.36</t>
         </is>
       </c>
       <c r="H24" s="14" t="inlineStr">

</xml_diff>